<commit_message>
fix(unifikasi): match Accounting Rp monetary display
</commit_message>
<xml_diff>
--- a/resources/unifikasi_format.xlsx
+++ b/resources/unifikasi_format.xlsx
@@ -381,7 +381,7 @@
     <ns0:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <ns0:xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </ns0:cellStyleXfs>
-  <ns0:cellXfs count="42">
+  <ns0:cellXfs count="44">
     <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -478,6 +478,10 @@
       <ns0:alignment vertical="top"/>
     </ns0:xf>
     <ns0:xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+      <ns0:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <ns0:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
       <ns0:alignment horizontal="center" vertical="top" wrapText="1"/>
     </ns0:xf>
   </ns0:cellXfs>
@@ -859,48 +863,48 @@
       <ns0:c r="B10" s="5" t="s">
         <ns0:v>16</ns0:v>
       </ns0:c>
-      <ns0:c r="C10" s="37"/>
-      <ns0:c r="D10" s="37"/>
-      <ns0:c r="E10" s="37"/>
-      <ns0:c r="F10" s="37"/>
-      <ns0:c r="G10" s="37"/>
-      <ns0:c r="H10" s="37"/>
+      <ns0:c r="C10" s="14"/>
+      <ns0:c r="D10" s="14"/>
+      <ns0:c r="E10" s="14"/>
+      <ns0:c r="F10" s="14"/>
+      <ns0:c r="G10" s="14"/>
+      <ns0:c r="H10" s="14"/>
     </ns0:row>
     <ns0:row r="11" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A11" s="3"/>
       <ns0:c r="B11" s="3" t="s">
         <ns0:v>17</ns0:v>
       </ns0:c>
-      <ns0:c r="C11" s="37"/>
-      <ns0:c r="D11" s="37"/>
-      <ns0:c r="E11" s="37"/>
-      <ns0:c r="F11" s="37"/>
-      <ns0:c r="G11" s="37"/>
-      <ns0:c r="H11" s="37"/>
+      <ns0:c r="C11" s="14"/>
+      <ns0:c r="D11" s="14"/>
+      <ns0:c r="E11" s="14"/>
+      <ns0:c r="F11" s="14"/>
+      <ns0:c r="G11" s="14"/>
+      <ns0:c r="H11" s="14"/>
     </ns0:row>
     <ns0:row r="12" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A12" s="3"/>
       <ns0:c r="B12" s="3" t="s">
         <ns0:v>18</ns0:v>
       </ns0:c>
-      <ns0:c r="C12" s="37"/>
-      <ns0:c r="D12" s="37"/>
-      <ns0:c r="E12" s="37"/>
-      <ns0:c r="F12" s="37"/>
-      <ns0:c r="G12" s="37"/>
-      <ns0:c r="H12" s="37"/>
+      <ns0:c r="C12" s="14"/>
+      <ns0:c r="D12" s="14"/>
+      <ns0:c r="E12" s="14"/>
+      <ns0:c r="F12" s="14"/>
+      <ns0:c r="G12" s="14"/>
+      <ns0:c r="H12" s="14"/>
     </ns0:row>
     <ns0:row r="13" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A13" s="3"/>
       <ns0:c r="B13" s="3" t="s">
         <ns0:v>19</ns0:v>
       </ns0:c>
-      <ns0:c r="C13" s="37"/>
-      <ns0:c r="D13" s="37"/>
-      <ns0:c r="E13" s="37"/>
-      <ns0:c r="F13" s="37"/>
-      <ns0:c r="G13" s="37"/>
-      <ns0:c r="H13" s="37"/>
+      <ns0:c r="C13" s="14"/>
+      <ns0:c r="D13" s="14"/>
+      <ns0:c r="E13" s="14"/>
+      <ns0:c r="F13" s="14"/>
+      <ns0:c r="G13" s="14"/>
+      <ns0:c r="H13" s="14"/>
     </ns0:row>
     <ns0:row r="14" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A14" s="5">
@@ -909,36 +913,36 @@
       <ns0:c r="B14" s="5" t="s">
         <ns0:v>20</ns0:v>
       </ns0:c>
-      <ns0:c r="C14" s="38"/>
-      <ns0:c r="D14" s="38"/>
-      <ns0:c r="E14" s="38"/>
-      <ns0:c r="F14" s="38"/>
-      <ns0:c r="G14" s="38"/>
-      <ns0:c r="H14" s="38"/>
+      <ns0:c r="C14" s="15"/>
+      <ns0:c r="D14" s="15"/>
+      <ns0:c r="E14" s="15"/>
+      <ns0:c r="F14" s="15"/>
+      <ns0:c r="G14" s="15"/>
+      <ns0:c r="H14" s="15"/>
     </ns0:row>
     <ns0:row r="15" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A15" s="3"/>
       <ns0:c r="B15" s="3" t="s">
         <ns0:v>21</ns0:v>
       </ns0:c>
-      <ns0:c r="C15" s="37"/>
-      <ns0:c r="D15" s="37"/>
-      <ns0:c r="E15" s="37"/>
-      <ns0:c r="F15" s="37"/>
-      <ns0:c r="G15" s="37"/>
-      <ns0:c r="H15" s="37"/>
+      <ns0:c r="C15" s="14"/>
+      <ns0:c r="D15" s="14"/>
+      <ns0:c r="E15" s="14"/>
+      <ns0:c r="F15" s="14"/>
+      <ns0:c r="G15" s="14"/>
+      <ns0:c r="H15" s="14"/>
     </ns0:row>
     <ns0:row r="16" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A16" s="3"/>
       <ns0:c r="B16" s="3" t="s">
         <ns0:v>22</ns0:v>
       </ns0:c>
-      <ns0:c r="C16" s="37"/>
-      <ns0:c r="D16" s="37"/>
-      <ns0:c r="E16" s="37"/>
-      <ns0:c r="F16" s="37"/>
-      <ns0:c r="G16" s="37"/>
-      <ns0:c r="H16" s="37"/>
+      <ns0:c r="C16" s="14"/>
+      <ns0:c r="D16" s="14"/>
+      <ns0:c r="E16" s="14"/>
+      <ns0:c r="F16" s="14"/>
+      <ns0:c r="G16" s="14"/>
+      <ns0:c r="H16" s="14"/>
     </ns0:row>
     <ns0:row r="17" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A17" s="5">
@@ -947,48 +951,48 @@
       <ns0:c r="B17" s="5" t="s">
         <ns0:v>23</ns0:v>
       </ns0:c>
-      <ns0:c r="C17" s="38"/>
-      <ns0:c r="D17" s="38"/>
-      <ns0:c r="E17" s="38"/>
-      <ns0:c r="F17" s="38"/>
-      <ns0:c r="G17" s="38"/>
-      <ns0:c r="H17" s="38"/>
+      <ns0:c r="C17" s="15"/>
+      <ns0:c r="D17" s="15"/>
+      <ns0:c r="E17" s="15"/>
+      <ns0:c r="F17" s="15"/>
+      <ns0:c r="G17" s="15"/>
+      <ns0:c r="H17" s="15"/>
     </ns0:row>
     <ns0:row r="18" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A18" s="3"/>
       <ns0:c r="B18" s="3" t="s">
         <ns0:v>24</ns0:v>
       </ns0:c>
-      <ns0:c r="C18" s="37"/>
-      <ns0:c r="D18" s="37"/>
-      <ns0:c r="E18" s="37"/>
-      <ns0:c r="F18" s="37"/>
-      <ns0:c r="G18" s="37"/>
-      <ns0:c r="H18" s="37"/>
+      <ns0:c r="C18" s="14"/>
+      <ns0:c r="D18" s="14"/>
+      <ns0:c r="E18" s="14"/>
+      <ns0:c r="F18" s="14"/>
+      <ns0:c r="G18" s="14"/>
+      <ns0:c r="H18" s="14"/>
     </ns0:row>
     <ns0:row r="19" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A19" s="3"/>
       <ns0:c r="B19" s="3" t="s">
         <ns0:v>25</ns0:v>
       </ns0:c>
-      <ns0:c r="C19" s="37"/>
-      <ns0:c r="D19" s="37"/>
-      <ns0:c r="E19" s="37"/>
-      <ns0:c r="F19" s="37"/>
-      <ns0:c r="G19" s="37"/>
-      <ns0:c r="H19" s="37"/>
+      <ns0:c r="C19" s="14"/>
+      <ns0:c r="D19" s="14"/>
+      <ns0:c r="E19" s="14"/>
+      <ns0:c r="F19" s="14"/>
+      <ns0:c r="G19" s="14"/>
+      <ns0:c r="H19" s="14"/>
     </ns0:row>
     <ns0:row r="20" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A20" s="3"/>
       <ns0:c r="B20" s="3" t="s">
         <ns0:v>26</ns0:v>
       </ns0:c>
-      <ns0:c r="C20" s="37"/>
-      <ns0:c r="D20" s="37"/>
-      <ns0:c r="E20" s="37"/>
-      <ns0:c r="F20" s="37"/>
-      <ns0:c r="G20" s="37"/>
-      <ns0:c r="H20" s="37"/>
+      <ns0:c r="C20" s="14"/>
+      <ns0:c r="D20" s="14"/>
+      <ns0:c r="E20" s="14"/>
+      <ns0:c r="F20" s="14"/>
+      <ns0:c r="G20" s="14"/>
+      <ns0:c r="H20" s="14"/>
     </ns0:row>
     <ns0:row r="21" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A21" s="5">
@@ -997,24 +1001,24 @@
       <ns0:c r="B21" s="5" t="s">
         <ns0:v>27</ns0:v>
       </ns0:c>
-      <ns0:c r="C21" s="38"/>
-      <ns0:c r="D21" s="38"/>
-      <ns0:c r="E21" s="38"/>
-      <ns0:c r="F21" s="38"/>
-      <ns0:c r="G21" s="38"/>
-      <ns0:c r="H21" s="38"/>
+      <ns0:c r="C21" s="15"/>
+      <ns0:c r="D21" s="15"/>
+      <ns0:c r="E21" s="15"/>
+      <ns0:c r="F21" s="15"/>
+      <ns0:c r="G21" s="15"/>
+      <ns0:c r="H21" s="15"/>
     </ns0:row>
     <ns0:row r="22" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A22" s="3"/>
       <ns0:c r="B22" s="3" t="s">
         <ns0:v>28</ns0:v>
       </ns0:c>
-      <ns0:c r="C22" s="37"/>
-      <ns0:c r="D22" s="37"/>
-      <ns0:c r="E22" s="37"/>
-      <ns0:c r="F22" s="37"/>
-      <ns0:c r="G22" s="37"/>
-      <ns0:c r="H22" s="37"/>
+      <ns0:c r="C22" s="14"/>
+      <ns0:c r="D22" s="14"/>
+      <ns0:c r="E22" s="14"/>
+      <ns0:c r="F22" s="14"/>
+      <ns0:c r="G22" s="14"/>
+      <ns0:c r="H22" s="14"/>
     </ns0:row>
     <ns0:row r="23" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A23" s="5">
@@ -1023,36 +1027,36 @@
       <ns0:c r="B23" s="5" t="s">
         <ns0:v>29</ns0:v>
       </ns0:c>
-      <ns0:c r="C23" s="38"/>
-      <ns0:c r="D23" s="38"/>
-      <ns0:c r="E23" s="38"/>
-      <ns0:c r="F23" s="38"/>
-      <ns0:c r="G23" s="38"/>
-      <ns0:c r="H23" s="38"/>
+      <ns0:c r="C23" s="15"/>
+      <ns0:c r="D23" s="15"/>
+      <ns0:c r="E23" s="15"/>
+      <ns0:c r="F23" s="15"/>
+      <ns0:c r="G23" s="15"/>
+      <ns0:c r="H23" s="15"/>
     </ns0:row>
     <ns0:row r="24" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A24" s="3"/>
       <ns0:c r="B24" s="3" t="s">
         <ns0:v>30</ns0:v>
       </ns0:c>
-      <ns0:c r="C24" s="37"/>
-      <ns0:c r="D24" s="37"/>
-      <ns0:c r="E24" s="37"/>
-      <ns0:c r="F24" s="37"/>
-      <ns0:c r="G24" s="37"/>
-      <ns0:c r="H24" s="37"/>
+      <ns0:c r="C24" s="14"/>
+      <ns0:c r="D24" s="14"/>
+      <ns0:c r="E24" s="14"/>
+      <ns0:c r="F24" s="14"/>
+      <ns0:c r="G24" s="14"/>
+      <ns0:c r="H24" s="14"/>
     </ns0:row>
     <ns0:row r="25" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A25" s="5" t="s">
         <ns0:v>31</ns0:v>
       </ns0:c>
       <ns0:c r="B25" s="5"/>
-      <ns0:c r="C25" s="38"/>
-      <ns0:c r="D25" s="38"/>
-      <ns0:c r="E25" s="38"/>
-      <ns0:c r="F25" s="38"/>
-      <ns0:c r="G25" s="38"/>
-      <ns0:c r="H25" s="38"/>
+      <ns0:c r="C25" s="15"/>
+      <ns0:c r="D25" s="15"/>
+      <ns0:c r="E25" s="15"/>
+      <ns0:c r="F25" s="15"/>
+      <ns0:c r="G25" s="15"/>
+      <ns0:c r="H25" s="15"/>
     </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells count="9">
@@ -1193,8 +1197,8 @@
       <ns0:c r="F5" s="17"/>
       <ns0:c r="G5" s="3"/>
       <ns0:c r="H5" s="18"/>
-      <ns0:c r="I5" s="37"/>
-      <ns0:c r="J5" s="37"/>
+      <ns0:c r="I5" s="14"/>
+      <ns0:c r="J5" s="14"/>
       <ns0:c r="K5" s="3"/>
       <ns0:c r="L5" s="3"/>
       <ns0:c r="M5" s="7"/>
@@ -1210,8 +1214,8 @@
       <ns0:c r="F6" s="17"/>
       <ns0:c r="G6" s="3"/>
       <ns0:c r="H6" s="18"/>
-      <ns0:c r="I6" s="37"/>
-      <ns0:c r="J6" s="37"/>
+      <ns0:c r="I6" s="14"/>
+      <ns0:c r="J6" s="14"/>
       <ns0:c r="K6" s="3"/>
       <ns0:c r="L6" s="3"/>
       <ns0:c r="M6" s="7"/>
@@ -1227,8 +1231,8 @@
       <ns0:c r="F7" s="17"/>
       <ns0:c r="G7" s="3"/>
       <ns0:c r="H7" s="18"/>
-      <ns0:c r="I7" s="37"/>
-      <ns0:c r="J7" s="37"/>
+      <ns0:c r="I7" s="14"/>
+      <ns0:c r="J7" s="14"/>
       <ns0:c r="K7" s="3"/>
       <ns0:c r="L7" s="3"/>
       <ns0:c r="M7" s="7"/>
@@ -1244,8 +1248,8 @@
       <ns0:c r="F8" s="17"/>
       <ns0:c r="G8" s="3"/>
       <ns0:c r="H8" s="18"/>
-      <ns0:c r="I8" s="37"/>
-      <ns0:c r="J8" s="37"/>
+      <ns0:c r="I8" s="14"/>
+      <ns0:c r="J8" s="14"/>
       <ns0:c r="K8" s="3"/>
       <ns0:c r="L8" s="3"/>
       <ns0:c r="M8" s="7"/>
@@ -1319,8 +1323,8 @@
       <ns0:c r="F11" s="17"/>
       <ns0:c r="G11" s="3"/>
       <ns0:c r="H11" s="18"/>
-      <ns0:c r="I11" s="37"/>
-      <ns0:c r="J11" s="37"/>
+      <ns0:c r="I11" s="14"/>
+      <ns0:c r="J11" s="14"/>
       <ns0:c r="K11" s="3"/>
       <ns0:c r="L11" s="3"/>
       <ns0:c r="M11" s="7"/>
@@ -1336,8 +1340,8 @@
       <ns0:c r="F12" s="17"/>
       <ns0:c r="G12" s="3"/>
       <ns0:c r="H12" s="18"/>
-      <ns0:c r="I12" s="37"/>
-      <ns0:c r="J12" s="37"/>
+      <ns0:c r="I12" s="14"/>
+      <ns0:c r="J12" s="14"/>
       <ns0:c r="K12" s="3"/>
       <ns0:c r="L12" s="3"/>
       <ns0:c r="M12" s="7"/>
@@ -1353,40 +1357,44 @@
       <ns0:c r="F13" s="17"/>
       <ns0:c r="G13" s="3"/>
       <ns0:c r="H13" s="18"/>
-      <ns0:c r="I13" s="37"/>
-      <ns0:c r="J13" s="37"/>
+      <ns0:c r="I13" s="14"/>
+      <ns0:c r="J13" s="14"/>
       <ns0:c r="K13" s="3"/>
       <ns0:c r="L13" s="3"/>
       <ns0:c r="M13" s="7"/>
       <ns0:c r="N13" s="3"/>
       <ns0:c r="O13" s="3"/>
     </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="I14" s="42"/>
+      <ns0:c r="J14" s="42"/>
+    </ns0:row>
     <ns0:row r="15" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A15" s="1" t="s">
         <ns0:v>52</ns0:v>
       </ns0:c>
       <ns0:c r="H15" s="8"/>
-      <ns0:c r="J15" s="39"/>
+      <ns0:c r="J15" s="19"/>
     </ns0:row>
     <ns0:row r="16" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A16" s="1" t="s">
         <ns0:v>53</ns0:v>
       </ns0:c>
       <ns0:c r="H16" s="8"/>
-      <ns0:c r="J16" s="39"/>
+      <ns0:c r="J16" s="19"/>
     </ns0:row>
     <ns0:row r="17" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A17" s="1" t="s">
         <ns0:v>54</ns0:v>
       </ns0:c>
       <ns0:c r="H17" s="8"/>
-      <ns0:c r="J17" s="39"/>
+      <ns0:c r="J17" s="19"/>
     </ns0:row>
     <ns0:row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A18" s="1" t="s">
         <ns0:v>55</ns0:v>
       </ns0:c>
-      <ns0:c r="J18" s="39"/>
+      <ns0:c r="J18" s="19"/>
     </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells count="1">
@@ -1492,7 +1500,7 @@
       <ns0:c r="D5" s="18"/>
       <ns0:c r="E5" s="24"/>
       <ns0:c r="F5" s="26"/>
-      <ns0:c r="G5" s="40"/>
+      <ns0:c r="G5" s="27"/>
       <ns0:c r="H5" s="20"/>
       <ns0:c r="I5" s="28"/>
       <ns0:c r="J5" s="20"/>
@@ -1505,7 +1513,7 @@
       <ns0:c r="D6" s="18"/>
       <ns0:c r="E6" s="24"/>
       <ns0:c r="F6" s="26"/>
-      <ns0:c r="G6" s="40"/>
+      <ns0:c r="G6" s="27"/>
       <ns0:c r="H6" s="20"/>
       <ns0:c r="I6" s="28"/>
       <ns0:c r="J6" s="20"/>
@@ -1518,19 +1526,22 @@
       <ns0:c r="D7" s="18"/>
       <ns0:c r="E7" s="24"/>
       <ns0:c r="F7" s="26"/>
-      <ns0:c r="G7" s="40"/>
+      <ns0:c r="G7" s="27"/>
       <ns0:c r="H7" s="20"/>
       <ns0:c r="I7" s="28"/>
       <ns0:c r="J7" s="20"/>
       <ns0:c r="K7" s="20"/>
     </ns0:row>
     <ns0:row r="8" spans="1:11" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <ns0:c r="E8" s="42"/>
+      <ns0:c r="G8" s="42"/>
       <ns0:c r="H8"/>
     </ns0:row>
     <ns0:row r="9" spans="1:11" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A9" s="1" t="s">
         <ns0:v>61</ns0:v>
       </ns0:c>
+      <ns0:c r="G9" s="42"/>
       <ns0:c r="H9"/>
       <ns0:c r="J9" s="19"/>
     </ns0:row>
@@ -1538,6 +1549,7 @@
       <ns0:c r="A10" s="1" t="s">
         <ns0:v>62</ns0:v>
       </ns0:c>
+      <ns0:c r="G10" s="42"/>
       <ns0:c r="H10"/>
       <ns0:c r="J10" s="19"/>
     </ns0:row>
@@ -1595,7 +1607,7 @@
       <ns0:c r="D14" s="18"/>
       <ns0:c r="E14" s="24"/>
       <ns0:c r="F14" s="26"/>
-      <ns0:c r="G14" s="40"/>
+      <ns0:c r="G14" s="27"/>
       <ns0:c r="H14" s="20"/>
       <ns0:c r="I14" s="28"/>
       <ns0:c r="J14" s="20"/>
@@ -1608,7 +1620,7 @@
       <ns0:c r="D15" s="18"/>
       <ns0:c r="E15" s="24"/>
       <ns0:c r="F15" s="26"/>
-      <ns0:c r="G15" s="40"/>
+      <ns0:c r="G15" s="27"/>
       <ns0:c r="H15" s="20"/>
       <ns0:c r="I15" s="28"/>
       <ns0:c r="J15" s="20"/>
@@ -1621,16 +1633,21 @@
       <ns0:c r="D16" s="18"/>
       <ns0:c r="E16" s="24"/>
       <ns0:c r="F16" s="26"/>
-      <ns0:c r="G16" s="40"/>
+      <ns0:c r="G16" s="27"/>
       <ns0:c r="H16" s="20"/>
       <ns0:c r="I16" s="28"/>
       <ns0:c r="J16" s="20"/>
       <ns0:c r="K16" s="20"/>
     </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="E17" s="42"/>
+      <ns0:c r="G17" s="42"/>
+    </ns0:row>
     <ns0:row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A18" s="1" t="s">
         <ns0:v>62</ns0:v>
       </ns0:c>
+      <ns0:c r="G18" s="42"/>
       <ns0:c r="H18" s="8"/>
       <ns0:c r="J18" s="19"/>
     </ns0:row>
@@ -1776,7 +1793,7 @@
       <ns0:c r="J5" s="23"/>
       <ns0:c r="K5" s="30"/>
       <ns0:c r="L5" s="26"/>
-      <ns0:c r="M5" s="40"/>
+      <ns0:c r="M5" s="27"/>
       <ns0:c r="N5" s="20"/>
       <ns0:c r="O5" s="28"/>
       <ns0:c r="P5" s="20"/>
@@ -1795,7 +1812,7 @@
       <ns0:c r="J6" s="23"/>
       <ns0:c r="K6" s="30"/>
       <ns0:c r="L6" s="26"/>
-      <ns0:c r="M6" s="40"/>
+      <ns0:c r="M6" s="27"/>
       <ns0:c r="N6" s="20"/>
       <ns0:c r="O6" s="28"/>
       <ns0:c r="P6" s="20"/>
@@ -1814,13 +1831,16 @@
       <ns0:c r="J7" s="23"/>
       <ns0:c r="K7" s="30"/>
       <ns0:c r="L7" s="26"/>
-      <ns0:c r="M7" s="40"/>
+      <ns0:c r="M7" s="27"/>
       <ns0:c r="N7" s="20"/>
       <ns0:c r="O7" s="28"/>
       <ns0:c r="P7" s="20"/>
       <ns0:c r="Q7" s="20"/>
     </ns0:row>
-    <ns0:row r="8" spans="1:17" s="1" customFormat="1" ns3:dyDescent="0.25"/>
+    <ns0:row r="8" spans="1:17" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <ns0:c r="K8" s="42"/>
+      <ns0:c r="M8" s="42"/>
+    </ns0:row>
     <ns0:row r="9" spans="1:17" ns3:dyDescent="0.25">
       <ns0:c r="A9" s="12"/>
       <ns0:c r="B9" s="12"/>
@@ -1832,9 +1852,9 @@
       <ns0:c r="H9" s="12"/>
       <ns0:c r="I9" s="12"/>
       <ns0:c r="J9" s="12"/>
-      <ns0:c r="K9" s="12"/>
+      <ns0:c r="K9" s="43"/>
       <ns0:c r="L9" s="12"/>
-      <ns0:c r="M9" s="41"/>
+      <ns0:c r="M9" s="43"/>
       <ns0:c r="N9" s="12"/>
     </ns0:row>
     <ns0:row r="10" spans="1:17" s="1" customFormat="1" ns3:dyDescent="0.25">
@@ -1842,7 +1862,7 @@
         <ns0:v>74</ns0:v>
       </ns0:c>
       <ns0:c r="G10" s="13"/>
-      <ns0:c r="M10" s="39"/>
+      <ns0:c r="M10" s="19"/>
     </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells count="1">

</xml_diff>

<commit_message>
fix(unifikasi): match PPN/PPh21 Accounting Rp formatting (#39)
* test(unifikasi): require Accounting Rp display parity

* fix(unifikasi): match Accounting Rp monetary display

---------

Co-authored-by: Punto Ami Priyono <189459396+cepeter@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resources/unifikasi_format.xlsx
+++ b/resources/unifikasi_format.xlsx
@@ -381,7 +381,7 @@
     <ns0:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <ns0:xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </ns0:cellStyleXfs>
-  <ns0:cellXfs count="42">
+  <ns0:cellXfs count="44">
     <ns0:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <ns0:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -478,6 +478,10 @@
       <ns0:alignment vertical="top"/>
     </ns0:xf>
     <ns0:xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
+      <ns0:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </ns0:xf>
+    <ns0:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <ns0:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyNumberFormat="1">
       <ns0:alignment horizontal="center" vertical="top" wrapText="1"/>
     </ns0:xf>
   </ns0:cellXfs>
@@ -859,48 +863,48 @@
       <ns0:c r="B10" s="5" t="s">
         <ns0:v>16</ns0:v>
       </ns0:c>
-      <ns0:c r="C10" s="37"/>
-      <ns0:c r="D10" s="37"/>
-      <ns0:c r="E10" s="37"/>
-      <ns0:c r="F10" s="37"/>
-      <ns0:c r="G10" s="37"/>
-      <ns0:c r="H10" s="37"/>
+      <ns0:c r="C10" s="14"/>
+      <ns0:c r="D10" s="14"/>
+      <ns0:c r="E10" s="14"/>
+      <ns0:c r="F10" s="14"/>
+      <ns0:c r="G10" s="14"/>
+      <ns0:c r="H10" s="14"/>
     </ns0:row>
     <ns0:row r="11" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A11" s="3"/>
       <ns0:c r="B11" s="3" t="s">
         <ns0:v>17</ns0:v>
       </ns0:c>
-      <ns0:c r="C11" s="37"/>
-      <ns0:c r="D11" s="37"/>
-      <ns0:c r="E11" s="37"/>
-      <ns0:c r="F11" s="37"/>
-      <ns0:c r="G11" s="37"/>
-      <ns0:c r="H11" s="37"/>
+      <ns0:c r="C11" s="14"/>
+      <ns0:c r="D11" s="14"/>
+      <ns0:c r="E11" s="14"/>
+      <ns0:c r="F11" s="14"/>
+      <ns0:c r="G11" s="14"/>
+      <ns0:c r="H11" s="14"/>
     </ns0:row>
     <ns0:row r="12" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A12" s="3"/>
       <ns0:c r="B12" s="3" t="s">
         <ns0:v>18</ns0:v>
       </ns0:c>
-      <ns0:c r="C12" s="37"/>
-      <ns0:c r="D12" s="37"/>
-      <ns0:c r="E12" s="37"/>
-      <ns0:c r="F12" s="37"/>
-      <ns0:c r="G12" s="37"/>
-      <ns0:c r="H12" s="37"/>
+      <ns0:c r="C12" s="14"/>
+      <ns0:c r="D12" s="14"/>
+      <ns0:c r="E12" s="14"/>
+      <ns0:c r="F12" s="14"/>
+      <ns0:c r="G12" s="14"/>
+      <ns0:c r="H12" s="14"/>
     </ns0:row>
     <ns0:row r="13" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A13" s="3"/>
       <ns0:c r="B13" s="3" t="s">
         <ns0:v>19</ns0:v>
       </ns0:c>
-      <ns0:c r="C13" s="37"/>
-      <ns0:c r="D13" s="37"/>
-      <ns0:c r="E13" s="37"/>
-      <ns0:c r="F13" s="37"/>
-      <ns0:c r="G13" s="37"/>
-      <ns0:c r="H13" s="37"/>
+      <ns0:c r="C13" s="14"/>
+      <ns0:c r="D13" s="14"/>
+      <ns0:c r="E13" s="14"/>
+      <ns0:c r="F13" s="14"/>
+      <ns0:c r="G13" s="14"/>
+      <ns0:c r="H13" s="14"/>
     </ns0:row>
     <ns0:row r="14" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A14" s="5">
@@ -909,36 +913,36 @@
       <ns0:c r="B14" s="5" t="s">
         <ns0:v>20</ns0:v>
       </ns0:c>
-      <ns0:c r="C14" s="38"/>
-      <ns0:c r="D14" s="38"/>
-      <ns0:c r="E14" s="38"/>
-      <ns0:c r="F14" s="38"/>
-      <ns0:c r="G14" s="38"/>
-      <ns0:c r="H14" s="38"/>
+      <ns0:c r="C14" s="15"/>
+      <ns0:c r="D14" s="15"/>
+      <ns0:c r="E14" s="15"/>
+      <ns0:c r="F14" s="15"/>
+      <ns0:c r="G14" s="15"/>
+      <ns0:c r="H14" s="15"/>
     </ns0:row>
     <ns0:row r="15" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A15" s="3"/>
       <ns0:c r="B15" s="3" t="s">
         <ns0:v>21</ns0:v>
       </ns0:c>
-      <ns0:c r="C15" s="37"/>
-      <ns0:c r="D15" s="37"/>
-      <ns0:c r="E15" s="37"/>
-      <ns0:c r="F15" s="37"/>
-      <ns0:c r="G15" s="37"/>
-      <ns0:c r="H15" s="37"/>
+      <ns0:c r="C15" s="14"/>
+      <ns0:c r="D15" s="14"/>
+      <ns0:c r="E15" s="14"/>
+      <ns0:c r="F15" s="14"/>
+      <ns0:c r="G15" s="14"/>
+      <ns0:c r="H15" s="14"/>
     </ns0:row>
     <ns0:row r="16" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A16" s="3"/>
       <ns0:c r="B16" s="3" t="s">
         <ns0:v>22</ns0:v>
       </ns0:c>
-      <ns0:c r="C16" s="37"/>
-      <ns0:c r="D16" s="37"/>
-      <ns0:c r="E16" s="37"/>
-      <ns0:c r="F16" s="37"/>
-      <ns0:c r="G16" s="37"/>
-      <ns0:c r="H16" s="37"/>
+      <ns0:c r="C16" s="14"/>
+      <ns0:c r="D16" s="14"/>
+      <ns0:c r="E16" s="14"/>
+      <ns0:c r="F16" s="14"/>
+      <ns0:c r="G16" s="14"/>
+      <ns0:c r="H16" s="14"/>
     </ns0:row>
     <ns0:row r="17" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A17" s="5">
@@ -947,48 +951,48 @@
       <ns0:c r="B17" s="5" t="s">
         <ns0:v>23</ns0:v>
       </ns0:c>
-      <ns0:c r="C17" s="38"/>
-      <ns0:c r="D17" s="38"/>
-      <ns0:c r="E17" s="38"/>
-      <ns0:c r="F17" s="38"/>
-      <ns0:c r="G17" s="38"/>
-      <ns0:c r="H17" s="38"/>
+      <ns0:c r="C17" s="15"/>
+      <ns0:c r="D17" s="15"/>
+      <ns0:c r="E17" s="15"/>
+      <ns0:c r="F17" s="15"/>
+      <ns0:c r="G17" s="15"/>
+      <ns0:c r="H17" s="15"/>
     </ns0:row>
     <ns0:row r="18" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A18" s="3"/>
       <ns0:c r="B18" s="3" t="s">
         <ns0:v>24</ns0:v>
       </ns0:c>
-      <ns0:c r="C18" s="37"/>
-      <ns0:c r="D18" s="37"/>
-      <ns0:c r="E18" s="37"/>
-      <ns0:c r="F18" s="37"/>
-      <ns0:c r="G18" s="37"/>
-      <ns0:c r="H18" s="37"/>
+      <ns0:c r="C18" s="14"/>
+      <ns0:c r="D18" s="14"/>
+      <ns0:c r="E18" s="14"/>
+      <ns0:c r="F18" s="14"/>
+      <ns0:c r="G18" s="14"/>
+      <ns0:c r="H18" s="14"/>
     </ns0:row>
     <ns0:row r="19" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A19" s="3"/>
       <ns0:c r="B19" s="3" t="s">
         <ns0:v>25</ns0:v>
       </ns0:c>
-      <ns0:c r="C19" s="37"/>
-      <ns0:c r="D19" s="37"/>
-      <ns0:c r="E19" s="37"/>
-      <ns0:c r="F19" s="37"/>
-      <ns0:c r="G19" s="37"/>
-      <ns0:c r="H19" s="37"/>
+      <ns0:c r="C19" s="14"/>
+      <ns0:c r="D19" s="14"/>
+      <ns0:c r="E19" s="14"/>
+      <ns0:c r="F19" s="14"/>
+      <ns0:c r="G19" s="14"/>
+      <ns0:c r="H19" s="14"/>
     </ns0:row>
     <ns0:row r="20" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A20" s="3"/>
       <ns0:c r="B20" s="3" t="s">
         <ns0:v>26</ns0:v>
       </ns0:c>
-      <ns0:c r="C20" s="37"/>
-      <ns0:c r="D20" s="37"/>
-      <ns0:c r="E20" s="37"/>
-      <ns0:c r="F20" s="37"/>
-      <ns0:c r="G20" s="37"/>
-      <ns0:c r="H20" s="37"/>
+      <ns0:c r="C20" s="14"/>
+      <ns0:c r="D20" s="14"/>
+      <ns0:c r="E20" s="14"/>
+      <ns0:c r="F20" s="14"/>
+      <ns0:c r="G20" s="14"/>
+      <ns0:c r="H20" s="14"/>
     </ns0:row>
     <ns0:row r="21" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A21" s="5">
@@ -997,24 +1001,24 @@
       <ns0:c r="B21" s="5" t="s">
         <ns0:v>27</ns0:v>
       </ns0:c>
-      <ns0:c r="C21" s="38"/>
-      <ns0:c r="D21" s="38"/>
-      <ns0:c r="E21" s="38"/>
-      <ns0:c r="F21" s="38"/>
-      <ns0:c r="G21" s="38"/>
-      <ns0:c r="H21" s="38"/>
+      <ns0:c r="C21" s="15"/>
+      <ns0:c r="D21" s="15"/>
+      <ns0:c r="E21" s="15"/>
+      <ns0:c r="F21" s="15"/>
+      <ns0:c r="G21" s="15"/>
+      <ns0:c r="H21" s="15"/>
     </ns0:row>
     <ns0:row r="22" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A22" s="3"/>
       <ns0:c r="B22" s="3" t="s">
         <ns0:v>28</ns0:v>
       </ns0:c>
-      <ns0:c r="C22" s="37"/>
-      <ns0:c r="D22" s="37"/>
-      <ns0:c r="E22" s="37"/>
-      <ns0:c r="F22" s="37"/>
-      <ns0:c r="G22" s="37"/>
-      <ns0:c r="H22" s="37"/>
+      <ns0:c r="C22" s="14"/>
+      <ns0:c r="D22" s="14"/>
+      <ns0:c r="E22" s="14"/>
+      <ns0:c r="F22" s="14"/>
+      <ns0:c r="G22" s="14"/>
+      <ns0:c r="H22" s="14"/>
     </ns0:row>
     <ns0:row r="23" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A23" s="5">
@@ -1023,36 +1027,36 @@
       <ns0:c r="B23" s="5" t="s">
         <ns0:v>29</ns0:v>
       </ns0:c>
-      <ns0:c r="C23" s="38"/>
-      <ns0:c r="D23" s="38"/>
-      <ns0:c r="E23" s="38"/>
-      <ns0:c r="F23" s="38"/>
-      <ns0:c r="G23" s="38"/>
-      <ns0:c r="H23" s="38"/>
+      <ns0:c r="C23" s="15"/>
+      <ns0:c r="D23" s="15"/>
+      <ns0:c r="E23" s="15"/>
+      <ns0:c r="F23" s="15"/>
+      <ns0:c r="G23" s="15"/>
+      <ns0:c r="H23" s="15"/>
     </ns0:row>
     <ns0:row r="24" spans="1:8" ns3:dyDescent="0.25">
       <ns0:c r="A24" s="3"/>
       <ns0:c r="B24" s="3" t="s">
         <ns0:v>30</ns0:v>
       </ns0:c>
-      <ns0:c r="C24" s="37"/>
-      <ns0:c r="D24" s="37"/>
-      <ns0:c r="E24" s="37"/>
-      <ns0:c r="F24" s="37"/>
-      <ns0:c r="G24" s="37"/>
-      <ns0:c r="H24" s="37"/>
+      <ns0:c r="C24" s="14"/>
+      <ns0:c r="D24" s="14"/>
+      <ns0:c r="E24" s="14"/>
+      <ns0:c r="F24" s="14"/>
+      <ns0:c r="G24" s="14"/>
+      <ns0:c r="H24" s="14"/>
     </ns0:row>
     <ns0:row r="25" spans="1:8" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A25" s="5" t="s">
         <ns0:v>31</ns0:v>
       </ns0:c>
       <ns0:c r="B25" s="5"/>
-      <ns0:c r="C25" s="38"/>
-      <ns0:c r="D25" s="38"/>
-      <ns0:c r="E25" s="38"/>
-      <ns0:c r="F25" s="38"/>
-      <ns0:c r="G25" s="38"/>
-      <ns0:c r="H25" s="38"/>
+      <ns0:c r="C25" s="15"/>
+      <ns0:c r="D25" s="15"/>
+      <ns0:c r="E25" s="15"/>
+      <ns0:c r="F25" s="15"/>
+      <ns0:c r="G25" s="15"/>
+      <ns0:c r="H25" s="15"/>
     </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells count="9">
@@ -1193,8 +1197,8 @@
       <ns0:c r="F5" s="17"/>
       <ns0:c r="G5" s="3"/>
       <ns0:c r="H5" s="18"/>
-      <ns0:c r="I5" s="37"/>
-      <ns0:c r="J5" s="37"/>
+      <ns0:c r="I5" s="14"/>
+      <ns0:c r="J5" s="14"/>
       <ns0:c r="K5" s="3"/>
       <ns0:c r="L5" s="3"/>
       <ns0:c r="M5" s="7"/>
@@ -1210,8 +1214,8 @@
       <ns0:c r="F6" s="17"/>
       <ns0:c r="G6" s="3"/>
       <ns0:c r="H6" s="18"/>
-      <ns0:c r="I6" s="37"/>
-      <ns0:c r="J6" s="37"/>
+      <ns0:c r="I6" s="14"/>
+      <ns0:c r="J6" s="14"/>
       <ns0:c r="K6" s="3"/>
       <ns0:c r="L6" s="3"/>
       <ns0:c r="M6" s="7"/>
@@ -1227,8 +1231,8 @@
       <ns0:c r="F7" s="17"/>
       <ns0:c r="G7" s="3"/>
       <ns0:c r="H7" s="18"/>
-      <ns0:c r="I7" s="37"/>
-      <ns0:c r="J7" s="37"/>
+      <ns0:c r="I7" s="14"/>
+      <ns0:c r="J7" s="14"/>
       <ns0:c r="K7" s="3"/>
       <ns0:c r="L7" s="3"/>
       <ns0:c r="M7" s="7"/>
@@ -1244,8 +1248,8 @@
       <ns0:c r="F8" s="17"/>
       <ns0:c r="G8" s="3"/>
       <ns0:c r="H8" s="18"/>
-      <ns0:c r="I8" s="37"/>
-      <ns0:c r="J8" s="37"/>
+      <ns0:c r="I8" s="14"/>
+      <ns0:c r="J8" s="14"/>
       <ns0:c r="K8" s="3"/>
       <ns0:c r="L8" s="3"/>
       <ns0:c r="M8" s="7"/>
@@ -1319,8 +1323,8 @@
       <ns0:c r="F11" s="17"/>
       <ns0:c r="G11" s="3"/>
       <ns0:c r="H11" s="18"/>
-      <ns0:c r="I11" s="37"/>
-      <ns0:c r="J11" s="37"/>
+      <ns0:c r="I11" s="14"/>
+      <ns0:c r="J11" s="14"/>
       <ns0:c r="K11" s="3"/>
       <ns0:c r="L11" s="3"/>
       <ns0:c r="M11" s="7"/>
@@ -1336,8 +1340,8 @@
       <ns0:c r="F12" s="17"/>
       <ns0:c r="G12" s="3"/>
       <ns0:c r="H12" s="18"/>
-      <ns0:c r="I12" s="37"/>
-      <ns0:c r="J12" s="37"/>
+      <ns0:c r="I12" s="14"/>
+      <ns0:c r="J12" s="14"/>
       <ns0:c r="K12" s="3"/>
       <ns0:c r="L12" s="3"/>
       <ns0:c r="M12" s="7"/>
@@ -1353,40 +1357,44 @@
       <ns0:c r="F13" s="17"/>
       <ns0:c r="G13" s="3"/>
       <ns0:c r="H13" s="18"/>
-      <ns0:c r="I13" s="37"/>
-      <ns0:c r="J13" s="37"/>
+      <ns0:c r="I13" s="14"/>
+      <ns0:c r="J13" s="14"/>
       <ns0:c r="K13" s="3"/>
       <ns0:c r="L13" s="3"/>
       <ns0:c r="M13" s="7"/>
       <ns0:c r="N13" s="3"/>
       <ns0:c r="O13" s="3"/>
     </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="I14" s="42"/>
+      <ns0:c r="J14" s="42"/>
+    </ns0:row>
     <ns0:row r="15" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A15" s="1" t="s">
         <ns0:v>52</ns0:v>
       </ns0:c>
       <ns0:c r="H15" s="8"/>
-      <ns0:c r="J15" s="39"/>
+      <ns0:c r="J15" s="19"/>
     </ns0:row>
     <ns0:row r="16" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A16" s="1" t="s">
         <ns0:v>53</ns0:v>
       </ns0:c>
       <ns0:c r="H16" s="8"/>
-      <ns0:c r="J16" s="39"/>
+      <ns0:c r="J16" s="19"/>
     </ns0:row>
     <ns0:row r="17" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A17" s="1" t="s">
         <ns0:v>54</ns0:v>
       </ns0:c>
       <ns0:c r="H17" s="8"/>
-      <ns0:c r="J17" s="39"/>
+      <ns0:c r="J17" s="19"/>
     </ns0:row>
     <ns0:row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A18" s="1" t="s">
         <ns0:v>55</ns0:v>
       </ns0:c>
-      <ns0:c r="J18" s="39"/>
+      <ns0:c r="J18" s="19"/>
     </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells count="1">
@@ -1492,7 +1500,7 @@
       <ns0:c r="D5" s="18"/>
       <ns0:c r="E5" s="24"/>
       <ns0:c r="F5" s="26"/>
-      <ns0:c r="G5" s="40"/>
+      <ns0:c r="G5" s="27"/>
       <ns0:c r="H5" s="20"/>
       <ns0:c r="I5" s="28"/>
       <ns0:c r="J5" s="20"/>
@@ -1505,7 +1513,7 @@
       <ns0:c r="D6" s="18"/>
       <ns0:c r="E6" s="24"/>
       <ns0:c r="F6" s="26"/>
-      <ns0:c r="G6" s="40"/>
+      <ns0:c r="G6" s="27"/>
       <ns0:c r="H6" s="20"/>
       <ns0:c r="I6" s="28"/>
       <ns0:c r="J6" s="20"/>
@@ -1518,19 +1526,22 @@
       <ns0:c r="D7" s="18"/>
       <ns0:c r="E7" s="24"/>
       <ns0:c r="F7" s="26"/>
-      <ns0:c r="G7" s="40"/>
+      <ns0:c r="G7" s="27"/>
       <ns0:c r="H7" s="20"/>
       <ns0:c r="I7" s="28"/>
       <ns0:c r="J7" s="20"/>
       <ns0:c r="K7" s="20"/>
     </ns0:row>
     <ns0:row r="8" spans="1:11" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <ns0:c r="E8" s="42"/>
+      <ns0:c r="G8" s="42"/>
       <ns0:c r="H8"/>
     </ns0:row>
     <ns0:row r="9" spans="1:11" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A9" s="1" t="s">
         <ns0:v>61</ns0:v>
       </ns0:c>
+      <ns0:c r="G9" s="42"/>
       <ns0:c r="H9"/>
       <ns0:c r="J9" s="19"/>
     </ns0:row>
@@ -1538,6 +1549,7 @@
       <ns0:c r="A10" s="1" t="s">
         <ns0:v>62</ns0:v>
       </ns0:c>
+      <ns0:c r="G10" s="42"/>
       <ns0:c r="H10"/>
       <ns0:c r="J10" s="19"/>
     </ns0:row>
@@ -1595,7 +1607,7 @@
       <ns0:c r="D14" s="18"/>
       <ns0:c r="E14" s="24"/>
       <ns0:c r="F14" s="26"/>
-      <ns0:c r="G14" s="40"/>
+      <ns0:c r="G14" s="27"/>
       <ns0:c r="H14" s="20"/>
       <ns0:c r="I14" s="28"/>
       <ns0:c r="J14" s="20"/>
@@ -1608,7 +1620,7 @@
       <ns0:c r="D15" s="18"/>
       <ns0:c r="E15" s="24"/>
       <ns0:c r="F15" s="26"/>
-      <ns0:c r="G15" s="40"/>
+      <ns0:c r="G15" s="27"/>
       <ns0:c r="H15" s="20"/>
       <ns0:c r="I15" s="28"/>
       <ns0:c r="J15" s="20"/>
@@ -1621,16 +1633,21 @@
       <ns0:c r="D16" s="18"/>
       <ns0:c r="E16" s="24"/>
       <ns0:c r="F16" s="26"/>
-      <ns0:c r="G16" s="40"/>
+      <ns0:c r="G16" s="27"/>
       <ns0:c r="H16" s="20"/>
       <ns0:c r="I16" s="28"/>
       <ns0:c r="J16" s="20"/>
       <ns0:c r="K16" s="20"/>
     </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="E17" s="42"/>
+      <ns0:c r="G17" s="42"/>
+    </ns0:row>
     <ns0:row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <ns0:c r="A18" s="1" t="s">
         <ns0:v>62</ns0:v>
       </ns0:c>
+      <ns0:c r="G18" s="42"/>
       <ns0:c r="H18" s="8"/>
       <ns0:c r="J18" s="19"/>
     </ns0:row>
@@ -1776,7 +1793,7 @@
       <ns0:c r="J5" s="23"/>
       <ns0:c r="K5" s="30"/>
       <ns0:c r="L5" s="26"/>
-      <ns0:c r="M5" s="40"/>
+      <ns0:c r="M5" s="27"/>
       <ns0:c r="N5" s="20"/>
       <ns0:c r="O5" s="28"/>
       <ns0:c r="P5" s="20"/>
@@ -1795,7 +1812,7 @@
       <ns0:c r="J6" s="23"/>
       <ns0:c r="K6" s="30"/>
       <ns0:c r="L6" s="26"/>
-      <ns0:c r="M6" s="40"/>
+      <ns0:c r="M6" s="27"/>
       <ns0:c r="N6" s="20"/>
       <ns0:c r="O6" s="28"/>
       <ns0:c r="P6" s="20"/>
@@ -1814,13 +1831,16 @@
       <ns0:c r="J7" s="23"/>
       <ns0:c r="K7" s="30"/>
       <ns0:c r="L7" s="26"/>
-      <ns0:c r="M7" s="40"/>
+      <ns0:c r="M7" s="27"/>
       <ns0:c r="N7" s="20"/>
       <ns0:c r="O7" s="28"/>
       <ns0:c r="P7" s="20"/>
       <ns0:c r="Q7" s="20"/>
     </ns0:row>
-    <ns0:row r="8" spans="1:17" s="1" customFormat="1" ns3:dyDescent="0.25"/>
+    <ns0:row r="8" spans="1:17" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <ns0:c r="K8" s="42"/>
+      <ns0:c r="M8" s="42"/>
+    </ns0:row>
     <ns0:row r="9" spans="1:17" ns3:dyDescent="0.25">
       <ns0:c r="A9" s="12"/>
       <ns0:c r="B9" s="12"/>
@@ -1832,9 +1852,9 @@
       <ns0:c r="H9" s="12"/>
       <ns0:c r="I9" s="12"/>
       <ns0:c r="J9" s="12"/>
-      <ns0:c r="K9" s="12"/>
+      <ns0:c r="K9" s="43"/>
       <ns0:c r="L9" s="12"/>
-      <ns0:c r="M9" s="41"/>
+      <ns0:c r="M9" s="43"/>
       <ns0:c r="N9" s="12"/>
     </ns0:row>
     <ns0:row r="10" spans="1:17" s="1" customFormat="1" ns3:dyDescent="0.25">
@@ -1842,7 +1862,7 @@
         <ns0:v>74</ns0:v>
       </ns0:c>
       <ns0:c r="G10" s="13"/>
-      <ns0:c r="M10" s="39"/>
+      <ns0:c r="M10" s="19"/>
     </ns0:row>
   </ns0:sheetData>
   <ns0:mergeCells count="1">

</xml_diff>

<commit_message>
fix: wait for PPN forms and recover Masa navigation with rate layout
</commit_message>
<xml_diff>
--- a/resources/unifikasi_format.xlsx
+++ b/resources/unifikasi_format.xlsx
@@ -1076,332 +1076,351 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{8B77BCAA-021F-44EB-B871-ECE64BD6C99A}">
-  <ns0:dimension ref="A1:O18"/>
-  <ns0:sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
-  <ns0:cols>
-    <ns0:col min="1" max="1" width="7.5703125" customWidth="1"/>
-    <ns0:col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <ns0:col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
-    <ns0:col min="4" max="4" width="17.7109375" customWidth="1"/>
-    <ns0:col min="5" max="5" width="16.140625" customWidth="1"/>
-    <ns0:col min="6" max="7" width="17.140625" customWidth="1"/>
-    <ns0:col min="8" max="8" width="19.28515625" customWidth="1"/>
-    <ns0:col min="9" max="9" width="14.140625" customWidth="1"/>
-    <ns0:col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
-    <ns0:col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
-    <ns0:col min="12" max="12" width="14.42578125" customWidth="1"/>
-    <ns0:col min="13" max="13" width="26.7109375" bestFit="1" customWidth="1"/>
-    <ns0:col min="14" max="14" width="11.42578125" customWidth="1"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1" spans="1:15" ns3:dyDescent="0.25">
-      <ns0:c r="A1" s="31" t="s">
-        <ns0:v>32</ns0:v>
-      </ns0:c>
-      <ns0:c r="B1" s="31"/>
-      <ns0:c r="C1" s="31"/>
-      <ns0:c r="D1" s="31"/>
-      <ns0:c r="E1" s="31"/>
-      <ns0:c r="F1" s="31"/>
-      <ns0:c r="G1" s="31"/>
-      <ns0:c r="H1" s="31"/>
-      <ns0:c r="I1" s="31"/>
-      <ns0:c r="J1" s="31"/>
-      <ns0:c r="K1" s="31"/>
-      <ns0:c r="L1" s="31"/>
-      <ns0:c r="M1" s="31"/>
-      <ns0:c r="N1" s="31"/>
-      <ns0:c r="O1" s="31"/>
-    </ns0:row>
-    <ns0:row r="2" spans="1:15" ns3:dyDescent="0.25">
-      <ns0:c r="A2" s="12"/>
-      <ns0:c r="B2" s="12"/>
-      <ns0:c r="C2" s="12"/>
-      <ns0:c r="D2" s="12"/>
-      <ns0:c r="E2" s="12"/>
-      <ns0:c r="F2" s="12"/>
-      <ns0:c r="G2" s="12"/>
-      <ns0:c r="H2" s="12"/>
-      <ns0:c r="I2" s="12"/>
-      <ns0:c r="J2" s="12"/>
-      <ns0:c r="K2" s="12"/>
-      <ns0:c r="L2" s="12"/>
-      <ns0:c r="M2" s="12"/>
-      <ns0:c r="N2" s="12"/>
-      <ns0:c r="O2" s="12"/>
-    </ns0:row>
-    <ns0:row r="3" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A3" s="1" t="s">
-        <ns0:v>33</ns0:v>
-      </ns0:c>
-      <ns0:c r="B3" s="1" t="s">
-        <ns0:v>34</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4" spans="1:15" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
-      <ns0:c r="A4" s="10" t="s">
-        <ns0:v>35</ns0:v>
-      </ns0:c>
-      <ns0:c r="B4" s="10" t="s">
-        <ns0:v>36</ns0:v>
-      </ns0:c>
-      <ns0:c r="C4" s="10" t="s">
-        <ns0:v>37</ns0:v>
-      </ns0:c>
-      <ns0:c r="D4" s="10" t="s">
-        <ns0:v>38</ns0:v>
-      </ns0:c>
-      <ns0:c r="E4" s="10" t="s">
-        <ns0:v>39</ns0:v>
-      </ns0:c>
-      <ns0:c r="F4" s="10" t="s">
-        <ns0:v>40</ns0:v>
-      </ns0:c>
-      <ns0:c r="G4" s="10" t="s">
-        <ns0:v>41</ns0:v>
-      </ns0:c>
-      <ns0:c r="H4" s="10" t="s">
-        <ns0:v>42</ns0:v>
-      </ns0:c>
-      <ns0:c r="I4" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>DASAR PENGENAAN PAJAK (Rp)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J4" s="10" t="s">
-        <ns0:v>44</ns0:v>
-      </ns0:c>
-      <ns0:c r="K4" s="10" t="s">
-        <ns0:v>45</ns0:v>
-      </ns0:c>
-      <ns0:c r="L4" s="10" t="s">
-        <ns0:v>46</ns0:v>
-      </ns0:c>
-      <ns0:c r="M4" s="10" t="s">
-        <ns0:v>47</ns0:v>
-      </ns0:c>
-      <ns0:c r="N4" s="10" t="s">
-        <ns0:v>48</ns0:v>
-      </ns0:c>
-      <ns0:c r="O4" s="10" t="s">
-        <ns0:v>49</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5" spans="1:15" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
-      <ns0:c r="A5" s="3"/>
-      <ns0:c r="B5" s="6"/>
-      <ns0:c r="C5" s="3"/>
-      <ns0:c r="D5" s="3"/>
-      <ns0:c r="E5" s="11"/>
-      <ns0:c r="F5" s="17"/>
-      <ns0:c r="G5" s="3"/>
-      <ns0:c r="H5" s="18"/>
-      <ns0:c r="I5" s="14"/>
-      <ns0:c r="J5" s="14"/>
-      <ns0:c r="K5" s="3"/>
-      <ns0:c r="L5" s="3"/>
-      <ns0:c r="M5" s="7"/>
-      <ns0:c r="N5" s="3"/>
-      <ns0:c r="O5" s="3"/>
-    </ns0:row>
-    <ns0:row r="6" spans="1:15" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
-      <ns0:c r="A6" s="3"/>
-      <ns0:c r="B6" s="6"/>
-      <ns0:c r="C6" s="3"/>
-      <ns0:c r="D6" s="3"/>
-      <ns0:c r="E6" s="11"/>
-      <ns0:c r="F6" s="17"/>
-      <ns0:c r="G6" s="3"/>
-      <ns0:c r="H6" s="18"/>
-      <ns0:c r="I6" s="14"/>
-      <ns0:c r="J6" s="14"/>
-      <ns0:c r="K6" s="3"/>
-      <ns0:c r="L6" s="3"/>
-      <ns0:c r="M6" s="7"/>
-      <ns0:c r="N6" s="3"/>
-      <ns0:c r="O6" s="3"/>
-    </ns0:row>
-    <ns0:row r="7" spans="1:15" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
-      <ns0:c r="A7" s="3"/>
-      <ns0:c r="B7" s="6"/>
-      <ns0:c r="C7" s="3"/>
-      <ns0:c r="D7" s="3"/>
-      <ns0:c r="E7" s="11"/>
-      <ns0:c r="F7" s="17"/>
-      <ns0:c r="G7" s="3"/>
-      <ns0:c r="H7" s="18"/>
-      <ns0:c r="I7" s="14"/>
-      <ns0:c r="J7" s="14"/>
-      <ns0:c r="K7" s="3"/>
-      <ns0:c r="L7" s="3"/>
-      <ns0:c r="M7" s="7"/>
-      <ns0:c r="N7" s="3"/>
-      <ns0:c r="O7" s="3"/>
-    </ns0:row>
-    <ns0:row r="8" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A8" s="3"/>
-      <ns0:c r="B8" s="6"/>
-      <ns0:c r="C8" s="3"/>
-      <ns0:c r="D8" s="3"/>
-      <ns0:c r="E8" s="11"/>
-      <ns0:c r="F8" s="17"/>
-      <ns0:c r="G8" s="3"/>
-      <ns0:c r="H8" s="18"/>
-      <ns0:c r="I8" s="14"/>
-      <ns0:c r="J8" s="14"/>
-      <ns0:c r="K8" s="3"/>
-      <ns0:c r="L8" s="3"/>
-      <ns0:c r="M8" s="7"/>
-      <ns0:c r="N8" s="3"/>
-      <ns0:c r="O8" s="3"/>
-    </ns0:row>
-    <ns0:row r="9" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A9" s="1" t="s">
-        <ns0:v>50</ns0:v>
-      </ns0:c>
-      <ns0:c r="B9" s="1" t="s">
-        <ns0:v>51</ns0:v>
-      </ns0:c>
-      <ns0:c r="H9"/>
-    </ns0:row>
-    <ns0:row r="10" spans="1:15" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
-      <ns0:c r="A10" s="10" t="s">
-        <ns0:v>35</ns0:v>
-      </ns0:c>
-      <ns0:c r="B10" s="10" t="s">
-        <ns0:v>36</ns0:v>
-      </ns0:c>
-      <ns0:c r="C10" s="10" t="s">
-        <ns0:v>37</ns0:v>
-      </ns0:c>
-      <ns0:c r="D10" s="10" t="s">
-        <ns0:v>38</ns0:v>
-      </ns0:c>
-      <ns0:c r="E10" s="10" t="s">
-        <ns0:v>39</ns0:v>
-      </ns0:c>
-      <ns0:c r="F10" s="10" t="s">
-        <ns0:v>40</ns0:v>
-      </ns0:c>
-      <ns0:c r="G10" s="10" t="s">
-        <ns0:v>41</ns0:v>
-      </ns0:c>
-      <ns0:c r="H10" s="10" t="s">
-        <ns0:v>42</ns0:v>
-      </ns0:c>
-      <ns0:c r="I10" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>DASAR PENGENAAN PAJAK (Rp)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J10" s="10" t="s">
-        <ns0:v>44</ns0:v>
-      </ns0:c>
-      <ns0:c r="K10" s="10" t="s">
-        <ns0:v>45</ns0:v>
-      </ns0:c>
-      <ns0:c r="L10" s="10" t="s">
-        <ns0:v>46</ns0:v>
-      </ns0:c>
-      <ns0:c r="M10" s="10" t="s">
-        <ns0:v>47</ns0:v>
-      </ns0:c>
-      <ns0:c r="N10" s="10" t="s">
-        <ns0:v>48</ns0:v>
-      </ns0:c>
-      <ns0:c r="O10" s="10" t="s">
-        <ns0:v>49</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11" spans="1:15" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
-      <ns0:c r="A11" s="3"/>
-      <ns0:c r="B11" s="6"/>
-      <ns0:c r="C11" s="3"/>
-      <ns0:c r="D11" s="3"/>
-      <ns0:c r="E11" s="11"/>
-      <ns0:c r="F11" s="17"/>
-      <ns0:c r="G11" s="3"/>
-      <ns0:c r="H11" s="18"/>
-      <ns0:c r="I11" s="14"/>
-      <ns0:c r="J11" s="14"/>
-      <ns0:c r="K11" s="3"/>
-      <ns0:c r="L11" s="3"/>
-      <ns0:c r="M11" s="7"/>
-      <ns0:c r="N11" s="3"/>
-      <ns0:c r="O11" s="3"/>
-    </ns0:row>
-    <ns0:row r="12" spans="1:15" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
-      <ns0:c r="A12" s="3"/>
-      <ns0:c r="B12" s="6"/>
-      <ns0:c r="C12" s="3"/>
-      <ns0:c r="D12" s="3"/>
-      <ns0:c r="E12" s="11"/>
-      <ns0:c r="F12" s="17"/>
-      <ns0:c r="G12" s="3"/>
-      <ns0:c r="H12" s="18"/>
-      <ns0:c r="I12" s="14"/>
-      <ns0:c r="J12" s="14"/>
-      <ns0:c r="K12" s="3"/>
-      <ns0:c r="L12" s="3"/>
-      <ns0:c r="M12" s="7"/>
-      <ns0:c r="N12" s="3"/>
-      <ns0:c r="O12" s="3"/>
-    </ns0:row>
-    <ns0:row r="13" spans="1:15" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
-      <ns0:c r="A13" s="3"/>
-      <ns0:c r="B13" s="6"/>
-      <ns0:c r="C13" s="3"/>
-      <ns0:c r="D13" s="3"/>
-      <ns0:c r="E13" s="11"/>
-      <ns0:c r="F13" s="17"/>
-      <ns0:c r="G13" s="3"/>
-      <ns0:c r="H13" s="18"/>
-      <ns0:c r="I13" s="14"/>
-      <ns0:c r="J13" s="14"/>
-      <ns0:c r="K13" s="3"/>
-      <ns0:c r="L13" s="3"/>
-      <ns0:c r="M13" s="7"/>
-      <ns0:c r="N13" s="3"/>
-      <ns0:c r="O13" s="3"/>
-    </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="I14" s="42"/>
-      <ns0:c r="J14" s="42"/>
-    </ns0:row>
-    <ns0:row r="15" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A15" s="1" t="s">
-        <ns0:v>52</ns0:v>
-      </ns0:c>
-      <ns0:c r="H15" s="8"/>
-      <ns0:c r="J15" s="19"/>
-    </ns0:row>
-    <ns0:row r="16" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A16" s="1" t="s">
-        <ns0:v>53</ns0:v>
-      </ns0:c>
-      <ns0:c r="H16" s="8"/>
-      <ns0:c r="J16" s="19"/>
-    </ns0:row>
-    <ns0:row r="17" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A17" s="1" t="s">
-        <ns0:v>54</ns0:v>
-      </ns0:c>
-      <ns0:c r="H17" s="8"/>
-      <ns0:c r="J17" s="19"/>
-    </ns0:row>
-    <ns0:row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A18" s="1" t="s">
-        <ns0:v>55</ns0:v>
-      </ns0:c>
-      <ns0:c r="J18" s="19"/>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:mergeCells count="1">
-    <ns0:mergeCell ref="A1:O1"/>
-  </ns0:mergeCells>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{8B77BCAA-021F-44EB-B871-ECE64BD6C99A}">
+  <dimension ref="A1:P18"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="19.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" customWidth="1"/>
+    <col min="14" max="14" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ns3:dyDescent="0.25">
+      <c r="A1" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+    </row>
+    <row r="2" spans="1:16" ns3:dyDescent="0.25">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+    </row>
+    <row r="3" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>DASAR PENGENAAN PAJAK (Rp)</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>TINGKAT (%)</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+    </row>
+    <row r="6" spans="1:16" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+    </row>
+    <row r="7" spans="1:16" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+    </row>
+    <row r="8" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+    </row>
+    <row r="9" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9"/>
+    </row>
+    <row r="10" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>DASAR PENGENAAN PAJAK (Rp)</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>TINGKAT (%)</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="N10" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O10" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="P10" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+    </row>
+    <row r="12" spans="1:16" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+    </row>
+    <row r="13" spans="1:16" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+    </row>
+    <row r="14">
+      <c r="I14" s="42"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="42"/>
+    </row>
+    <row r="15" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H15" s="8"/>
+      <c r="K15" s="19"/>
+    </row>
+    <row r="16" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H16" s="8"/>
+      <c r="K16" s="19"/>
+    </row>
+    <row r="17" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" s="8"/>
+      <c r="K17" s="19"/>
+    </row>
+    <row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K18" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:P1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
fix: Masa capture readiness, navigation and Unifikasi layout (#43)
* test: pin PPN readiness and Unifikasi rate layout contracts

* test: exercise real paginator guards and failed panel recovery

* fix: wait for PPN forms and recover Masa navigation with rate layout

* test: clear static review findings and record runner acceptance

---------

Co-authored-by: Punto Ami Priyono <189459396+cepeter@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resources/unifikasi_format.xlsx
+++ b/resources/unifikasi_format.xlsx
@@ -1076,332 +1076,351 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{8B77BCAA-021F-44EB-B871-ECE64BD6C99A}">
-  <ns0:dimension ref="A1:O18"/>
-  <ns0:sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
-  <ns0:cols>
-    <ns0:col min="1" max="1" width="7.5703125" customWidth="1"/>
-    <ns0:col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <ns0:col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
-    <ns0:col min="4" max="4" width="17.7109375" customWidth="1"/>
-    <ns0:col min="5" max="5" width="16.140625" customWidth="1"/>
-    <ns0:col min="6" max="7" width="17.140625" customWidth="1"/>
-    <ns0:col min="8" max="8" width="19.28515625" customWidth="1"/>
-    <ns0:col min="9" max="9" width="14.140625" customWidth="1"/>
-    <ns0:col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
-    <ns0:col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
-    <ns0:col min="12" max="12" width="14.42578125" customWidth="1"/>
-    <ns0:col min="13" max="13" width="26.7109375" bestFit="1" customWidth="1"/>
-    <ns0:col min="14" max="14" width="11.42578125" customWidth="1"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1" spans="1:15" ns3:dyDescent="0.25">
-      <ns0:c r="A1" s="31" t="s">
-        <ns0:v>32</ns0:v>
-      </ns0:c>
-      <ns0:c r="B1" s="31"/>
-      <ns0:c r="C1" s="31"/>
-      <ns0:c r="D1" s="31"/>
-      <ns0:c r="E1" s="31"/>
-      <ns0:c r="F1" s="31"/>
-      <ns0:c r="G1" s="31"/>
-      <ns0:c r="H1" s="31"/>
-      <ns0:c r="I1" s="31"/>
-      <ns0:c r="J1" s="31"/>
-      <ns0:c r="K1" s="31"/>
-      <ns0:c r="L1" s="31"/>
-      <ns0:c r="M1" s="31"/>
-      <ns0:c r="N1" s="31"/>
-      <ns0:c r="O1" s="31"/>
-    </ns0:row>
-    <ns0:row r="2" spans="1:15" ns3:dyDescent="0.25">
-      <ns0:c r="A2" s="12"/>
-      <ns0:c r="B2" s="12"/>
-      <ns0:c r="C2" s="12"/>
-      <ns0:c r="D2" s="12"/>
-      <ns0:c r="E2" s="12"/>
-      <ns0:c r="F2" s="12"/>
-      <ns0:c r="G2" s="12"/>
-      <ns0:c r="H2" s="12"/>
-      <ns0:c r="I2" s="12"/>
-      <ns0:c r="J2" s="12"/>
-      <ns0:c r="K2" s="12"/>
-      <ns0:c r="L2" s="12"/>
-      <ns0:c r="M2" s="12"/>
-      <ns0:c r="N2" s="12"/>
-      <ns0:c r="O2" s="12"/>
-    </ns0:row>
-    <ns0:row r="3" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A3" s="1" t="s">
-        <ns0:v>33</ns0:v>
-      </ns0:c>
-      <ns0:c r="B3" s="1" t="s">
-        <ns0:v>34</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4" spans="1:15" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
-      <ns0:c r="A4" s="10" t="s">
-        <ns0:v>35</ns0:v>
-      </ns0:c>
-      <ns0:c r="B4" s="10" t="s">
-        <ns0:v>36</ns0:v>
-      </ns0:c>
-      <ns0:c r="C4" s="10" t="s">
-        <ns0:v>37</ns0:v>
-      </ns0:c>
-      <ns0:c r="D4" s="10" t="s">
-        <ns0:v>38</ns0:v>
-      </ns0:c>
-      <ns0:c r="E4" s="10" t="s">
-        <ns0:v>39</ns0:v>
-      </ns0:c>
-      <ns0:c r="F4" s="10" t="s">
-        <ns0:v>40</ns0:v>
-      </ns0:c>
-      <ns0:c r="G4" s="10" t="s">
-        <ns0:v>41</ns0:v>
-      </ns0:c>
-      <ns0:c r="H4" s="10" t="s">
-        <ns0:v>42</ns0:v>
-      </ns0:c>
-      <ns0:c r="I4" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>DASAR PENGENAAN PAJAK (Rp)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J4" s="10" t="s">
-        <ns0:v>44</ns0:v>
-      </ns0:c>
-      <ns0:c r="K4" s="10" t="s">
-        <ns0:v>45</ns0:v>
-      </ns0:c>
-      <ns0:c r="L4" s="10" t="s">
-        <ns0:v>46</ns0:v>
-      </ns0:c>
-      <ns0:c r="M4" s="10" t="s">
-        <ns0:v>47</ns0:v>
-      </ns0:c>
-      <ns0:c r="N4" s="10" t="s">
-        <ns0:v>48</ns0:v>
-      </ns0:c>
-      <ns0:c r="O4" s="10" t="s">
-        <ns0:v>49</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5" spans="1:15" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
-      <ns0:c r="A5" s="3"/>
-      <ns0:c r="B5" s="6"/>
-      <ns0:c r="C5" s="3"/>
-      <ns0:c r="D5" s="3"/>
-      <ns0:c r="E5" s="11"/>
-      <ns0:c r="F5" s="17"/>
-      <ns0:c r="G5" s="3"/>
-      <ns0:c r="H5" s="18"/>
-      <ns0:c r="I5" s="14"/>
-      <ns0:c r="J5" s="14"/>
-      <ns0:c r="K5" s="3"/>
-      <ns0:c r="L5" s="3"/>
-      <ns0:c r="M5" s="7"/>
-      <ns0:c r="N5" s="3"/>
-      <ns0:c r="O5" s="3"/>
-    </ns0:row>
-    <ns0:row r="6" spans="1:15" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
-      <ns0:c r="A6" s="3"/>
-      <ns0:c r="B6" s="6"/>
-      <ns0:c r="C6" s="3"/>
-      <ns0:c r="D6" s="3"/>
-      <ns0:c r="E6" s="11"/>
-      <ns0:c r="F6" s="17"/>
-      <ns0:c r="G6" s="3"/>
-      <ns0:c r="H6" s="18"/>
-      <ns0:c r="I6" s="14"/>
-      <ns0:c r="J6" s="14"/>
-      <ns0:c r="K6" s="3"/>
-      <ns0:c r="L6" s="3"/>
-      <ns0:c r="M6" s="7"/>
-      <ns0:c r="N6" s="3"/>
-      <ns0:c r="O6" s="3"/>
-    </ns0:row>
-    <ns0:row r="7" spans="1:15" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
-      <ns0:c r="A7" s="3"/>
-      <ns0:c r="B7" s="6"/>
-      <ns0:c r="C7" s="3"/>
-      <ns0:c r="D7" s="3"/>
-      <ns0:c r="E7" s="11"/>
-      <ns0:c r="F7" s="17"/>
-      <ns0:c r="G7" s="3"/>
-      <ns0:c r="H7" s="18"/>
-      <ns0:c r="I7" s="14"/>
-      <ns0:c r="J7" s="14"/>
-      <ns0:c r="K7" s="3"/>
-      <ns0:c r="L7" s="3"/>
-      <ns0:c r="M7" s="7"/>
-      <ns0:c r="N7" s="3"/>
-      <ns0:c r="O7" s="3"/>
-    </ns0:row>
-    <ns0:row r="8" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A8" s="3"/>
-      <ns0:c r="B8" s="6"/>
-      <ns0:c r="C8" s="3"/>
-      <ns0:c r="D8" s="3"/>
-      <ns0:c r="E8" s="11"/>
-      <ns0:c r="F8" s="17"/>
-      <ns0:c r="G8" s="3"/>
-      <ns0:c r="H8" s="18"/>
-      <ns0:c r="I8" s="14"/>
-      <ns0:c r="J8" s="14"/>
-      <ns0:c r="K8" s="3"/>
-      <ns0:c r="L8" s="3"/>
-      <ns0:c r="M8" s="7"/>
-      <ns0:c r="N8" s="3"/>
-      <ns0:c r="O8" s="3"/>
-    </ns0:row>
-    <ns0:row r="9" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A9" s="1" t="s">
-        <ns0:v>50</ns0:v>
-      </ns0:c>
-      <ns0:c r="B9" s="1" t="s">
-        <ns0:v>51</ns0:v>
-      </ns0:c>
-      <ns0:c r="H9"/>
-    </ns0:row>
-    <ns0:row r="10" spans="1:15" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
-      <ns0:c r="A10" s="10" t="s">
-        <ns0:v>35</ns0:v>
-      </ns0:c>
-      <ns0:c r="B10" s="10" t="s">
-        <ns0:v>36</ns0:v>
-      </ns0:c>
-      <ns0:c r="C10" s="10" t="s">
-        <ns0:v>37</ns0:v>
-      </ns0:c>
-      <ns0:c r="D10" s="10" t="s">
-        <ns0:v>38</ns0:v>
-      </ns0:c>
-      <ns0:c r="E10" s="10" t="s">
-        <ns0:v>39</ns0:v>
-      </ns0:c>
-      <ns0:c r="F10" s="10" t="s">
-        <ns0:v>40</ns0:v>
-      </ns0:c>
-      <ns0:c r="G10" s="10" t="s">
-        <ns0:v>41</ns0:v>
-      </ns0:c>
-      <ns0:c r="H10" s="10" t="s">
-        <ns0:v>42</ns0:v>
-      </ns0:c>
-      <ns0:c r="I10" s="10" t="inlineStr">
-        <ns0:is>
-          <ns0:t>DASAR PENGENAAN PAJAK (Rp)</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J10" s="10" t="s">
-        <ns0:v>44</ns0:v>
-      </ns0:c>
-      <ns0:c r="K10" s="10" t="s">
-        <ns0:v>45</ns0:v>
-      </ns0:c>
-      <ns0:c r="L10" s="10" t="s">
-        <ns0:v>46</ns0:v>
-      </ns0:c>
-      <ns0:c r="M10" s="10" t="s">
-        <ns0:v>47</ns0:v>
-      </ns0:c>
-      <ns0:c r="N10" s="10" t="s">
-        <ns0:v>48</ns0:v>
-      </ns0:c>
-      <ns0:c r="O10" s="10" t="s">
-        <ns0:v>49</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11" spans="1:15" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
-      <ns0:c r="A11" s="3"/>
-      <ns0:c r="B11" s="6"/>
-      <ns0:c r="C11" s="3"/>
-      <ns0:c r="D11" s="3"/>
-      <ns0:c r="E11" s="11"/>
-      <ns0:c r="F11" s="17"/>
-      <ns0:c r="G11" s="3"/>
-      <ns0:c r="H11" s="18"/>
-      <ns0:c r="I11" s="14"/>
-      <ns0:c r="J11" s="14"/>
-      <ns0:c r="K11" s="3"/>
-      <ns0:c r="L11" s="3"/>
-      <ns0:c r="M11" s="7"/>
-      <ns0:c r="N11" s="3"/>
-      <ns0:c r="O11" s="3"/>
-    </ns0:row>
-    <ns0:row r="12" spans="1:15" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
-      <ns0:c r="A12" s="3"/>
-      <ns0:c r="B12" s="6"/>
-      <ns0:c r="C12" s="3"/>
-      <ns0:c r="D12" s="3"/>
-      <ns0:c r="E12" s="11"/>
-      <ns0:c r="F12" s="17"/>
-      <ns0:c r="G12" s="3"/>
-      <ns0:c r="H12" s="18"/>
-      <ns0:c r="I12" s="14"/>
-      <ns0:c r="J12" s="14"/>
-      <ns0:c r="K12" s="3"/>
-      <ns0:c r="L12" s="3"/>
-      <ns0:c r="M12" s="7"/>
-      <ns0:c r="N12" s="3"/>
-      <ns0:c r="O12" s="3"/>
-    </ns0:row>
-    <ns0:row r="13" spans="1:15" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
-      <ns0:c r="A13" s="3"/>
-      <ns0:c r="B13" s="6"/>
-      <ns0:c r="C13" s="3"/>
-      <ns0:c r="D13" s="3"/>
-      <ns0:c r="E13" s="11"/>
-      <ns0:c r="F13" s="17"/>
-      <ns0:c r="G13" s="3"/>
-      <ns0:c r="H13" s="18"/>
-      <ns0:c r="I13" s="14"/>
-      <ns0:c r="J13" s="14"/>
-      <ns0:c r="K13" s="3"/>
-      <ns0:c r="L13" s="3"/>
-      <ns0:c r="M13" s="7"/>
-      <ns0:c r="N13" s="3"/>
-      <ns0:c r="O13" s="3"/>
-    </ns0:row>
-    <ns0:row r="14">
-      <ns0:c r="I14" s="42"/>
-      <ns0:c r="J14" s="42"/>
-    </ns0:row>
-    <ns0:row r="15" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A15" s="1" t="s">
-        <ns0:v>52</ns0:v>
-      </ns0:c>
-      <ns0:c r="H15" s="8"/>
-      <ns0:c r="J15" s="19"/>
-    </ns0:row>
-    <ns0:row r="16" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A16" s="1" t="s">
-        <ns0:v>53</ns0:v>
-      </ns0:c>
-      <ns0:c r="H16" s="8"/>
-      <ns0:c r="J16" s="19"/>
-    </ns0:row>
-    <ns0:row r="17" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A17" s="1" t="s">
-        <ns0:v>54</ns0:v>
-      </ns0:c>
-      <ns0:c r="H17" s="8"/>
-      <ns0:c r="J17" s="19"/>
-    </ns0:row>
-    <ns0:row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <ns0:c r="A18" s="1" t="s">
-        <ns0:v>55</ns0:v>
-      </ns0:c>
-      <ns0:c r="J18" s="19"/>
-    </ns0:row>
-  </ns0:sheetData>
-  <ns0:mergeCells count="1">
-    <ns0:mergeCell ref="A1:O1"/>
-  </ns0:mergeCells>
-  <ns0:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{8B77BCAA-021F-44EB-B871-ECE64BD6C99A}">
+  <dimension ref="A1:P18"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.140625" customWidth="1"/>
+    <col min="6" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="19.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" customWidth="1"/>
+    <col min="14" max="14" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ns3:dyDescent="0.25">
+      <c r="A1" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+    </row>
+    <row r="2" spans="1:16" ns3:dyDescent="0.25">
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+    </row>
+    <row r="3" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>DASAR PENGENAAN PAJAK (Rp)</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>TINGKAT (%)</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="N4" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+    </row>
+    <row r="6" spans="1:16" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+    </row>
+    <row r="7" spans="1:16" s="1" customFormat="1" ht="30" ns3:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+    </row>
+    <row r="8" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="14"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="14"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+    </row>
+    <row r="9" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9"/>
+    </row>
+    <row r="10" spans="1:16" s="9" customFormat="1" ht="47.25" customHeight="1" ns3:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>DASAR PENGENAAN PAJAK (Rp)</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>TINGKAT (%)</t>
+        </is>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M10" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="N10" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O10" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="P10" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+    </row>
+    <row r="12" spans="1:16" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+    </row>
+    <row r="13" spans="1:16" s="1" customFormat="1" ht="60" ns3:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="14"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+    </row>
+    <row r="14">
+      <c r="I14" s="42"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="42"/>
+    </row>
+    <row r="15" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H15" s="8"/>
+      <c r="K15" s="19"/>
+    </row>
+    <row r="16" spans="1:16" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H16" s="8"/>
+      <c r="K16" s="19"/>
+    </row>
+    <row r="17" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" s="8"/>
+      <c r="K17" s="19"/>
+    </row>
+    <row r="18" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K18" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:P1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>